<commit_message>
AGENT-1: revert Phase-1 mastery inversion to faithful original
Restore learning-system.xlsx Phase-1 H10:H39 to the original
=IFERROR(F/E*(1+G),0) (rewards higher mastery — intentional spaced-rep
design: mastered cards stay in high-priority quick-review rotation).
Fix SUPERLEARN-SPEC.md §1 (formula is correct as-is; tell AGENT-3 not to
invert) and §5.2 admission-order wording (domain Importance/Challenge;
mastery term is moot for never-started candidates). 414/414 cells eval clean.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/learning-system.xlsx
+++ b/learning-system.xlsx
@@ -627,7 +627,7 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5">
-        <f>IFERROR(F10/E10*(1+(1-G10)),0)</f>
+        <f>IFERROR(F10/E10*(1+G10),0)</f>
         <v/>
       </c>
     </row>
@@ -640,7 +640,7 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5">
-        <f>IFERROR(F11/E11*(1+(1-G11)),0)</f>
+        <f>IFERROR(F11/E11*(1+G11),0)</f>
         <v/>
       </c>
     </row>
@@ -653,7 +653,7 @@
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
       <c r="H12" s="5">
-        <f>IFERROR(F12/E12*(1+(1-G12)),0)</f>
+        <f>IFERROR(F12/E12*(1+G12),0)</f>
         <v/>
       </c>
     </row>
@@ -666,7 +666,7 @@
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5">
-        <f>IFERROR(F13/E13*(1+(1-G13)),0)</f>
+        <f>IFERROR(F13/E13*(1+G13),0)</f>
         <v/>
       </c>
     </row>
@@ -679,7 +679,7 @@
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5">
-        <f>IFERROR(F14/E14*(1+(1-G14)),0)</f>
+        <f>IFERROR(F14/E14*(1+G14),0)</f>
         <v/>
       </c>
     </row>
@@ -692,7 +692,7 @@
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5">
-        <f>IFERROR(F15/E15*(1+(1-G15)),0)</f>
+        <f>IFERROR(F15/E15*(1+G15),0)</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5">
-        <f>IFERROR(F16/E16*(1+(1-G16)),0)</f>
+        <f>IFERROR(F16/E16*(1+G16),0)</f>
         <v/>
       </c>
     </row>
@@ -718,7 +718,7 @@
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
       <c r="H17" s="5">
-        <f>IFERROR(F17/E17*(1+(1-G17)),0)</f>
+        <f>IFERROR(F17/E17*(1+G17),0)</f>
         <v/>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
       <c r="H18" s="5">
-        <f>IFERROR(F18/E18*(1+(1-G18)),0)</f>
+        <f>IFERROR(F18/E18*(1+G18),0)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
       <c r="H19" s="5">
-        <f>IFERROR(F19/E19*(1+(1-G19)),0)</f>
+        <f>IFERROR(F19/E19*(1+G19),0)</f>
         <v/>
       </c>
     </row>
@@ -757,7 +757,7 @@
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="5">
-        <f>IFERROR(F20/E20*(1+(1-G20)),0)</f>
+        <f>IFERROR(F20/E20*(1+G20),0)</f>
         <v/>
       </c>
     </row>
@@ -770,7 +770,7 @@
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
       <c r="H21" s="5">
-        <f>IFERROR(F21/E21*(1+(1-G21)),0)</f>
+        <f>IFERROR(F21/E21*(1+G21),0)</f>
         <v/>
       </c>
     </row>
@@ -783,7 +783,7 @@
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
       <c r="H22" s="5">
-        <f>IFERROR(F22/E22*(1+(1-G22)),0)</f>
+        <f>IFERROR(F22/E22*(1+G22),0)</f>
         <v/>
       </c>
     </row>
@@ -796,7 +796,7 @@
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
       <c r="H23" s="5">
-        <f>IFERROR(F23/E23*(1+(1-G23)),0)</f>
+        <f>IFERROR(F23/E23*(1+G23),0)</f>
         <v/>
       </c>
     </row>
@@ -809,7 +809,7 @@
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
       <c r="H24" s="5">
-        <f>IFERROR(F24/E24*(1+(1-G24)),0)</f>
+        <f>IFERROR(F24/E24*(1+G24),0)</f>
         <v/>
       </c>
     </row>
@@ -822,7 +822,7 @@
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
       <c r="H25" s="5">
-        <f>IFERROR(F25/E25*(1+(1-G25)),0)</f>
+        <f>IFERROR(F25/E25*(1+G25),0)</f>
         <v/>
       </c>
     </row>
@@ -835,7 +835,7 @@
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
       <c r="H26" s="5">
-        <f>IFERROR(F26/E26*(1+(1-G26)),0)</f>
+        <f>IFERROR(F26/E26*(1+G26),0)</f>
         <v/>
       </c>
     </row>
@@ -848,7 +848,7 @@
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="5" t="n"/>
       <c r="H27" s="5">
-        <f>IFERROR(F27/E27*(1+(1-G27)),0)</f>
+        <f>IFERROR(F27/E27*(1+G27),0)</f>
         <v/>
       </c>
     </row>
@@ -861,7 +861,7 @@
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
       <c r="H28" s="5">
-        <f>IFERROR(F28/E28*(1+(1-G28)),0)</f>
+        <f>IFERROR(F28/E28*(1+G28),0)</f>
         <v/>
       </c>
     </row>
@@ -874,7 +874,7 @@
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>
       <c r="H29" s="5">
-        <f>IFERROR(F29/E29*(1+(1-G29)),0)</f>
+        <f>IFERROR(F29/E29*(1+G29),0)</f>
         <v/>
       </c>
     </row>
@@ -887,7 +887,7 @@
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
       <c r="H30" s="5">
-        <f>IFERROR(F30/E30*(1+(1-G30)),0)</f>
+        <f>IFERROR(F30/E30*(1+G30),0)</f>
         <v/>
       </c>
     </row>
@@ -900,7 +900,7 @@
       <c r="F31" s="5" t="n"/>
       <c r="G31" s="5" t="n"/>
       <c r="H31" s="5">
-        <f>IFERROR(F31/E31*(1+(1-G31)),0)</f>
+        <f>IFERROR(F31/E31*(1+G31),0)</f>
         <v/>
       </c>
     </row>
@@ -913,7 +913,7 @@
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="5" t="n"/>
       <c r="H32" s="5">
-        <f>IFERROR(F32/E32*(1+(1-G32)),0)</f>
+        <f>IFERROR(F32/E32*(1+G32),0)</f>
         <v/>
       </c>
     </row>
@@ -926,7 +926,7 @@
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
       <c r="H33" s="5">
-        <f>IFERROR(F33/E33*(1+(1-G33)),0)</f>
+        <f>IFERROR(F33/E33*(1+G33),0)</f>
         <v/>
       </c>
     </row>
@@ -939,7 +939,7 @@
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="5" t="n"/>
       <c r="H34" s="5">
-        <f>IFERROR(F34/E34*(1+(1-G34)),0)</f>
+        <f>IFERROR(F34/E34*(1+G34),0)</f>
         <v/>
       </c>
     </row>
@@ -952,7 +952,7 @@
       <c r="F35" s="5" t="n"/>
       <c r="G35" s="5" t="n"/>
       <c r="H35" s="5">
-        <f>IFERROR(F35/E35*(1+(1-G35)),0)</f>
+        <f>IFERROR(F35/E35*(1+G35),0)</f>
         <v/>
       </c>
     </row>
@@ -965,7 +965,7 @@
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="5" t="n"/>
       <c r="H36" s="5">
-        <f>IFERROR(F36/E36*(1+(1-G36)),0)</f>
+        <f>IFERROR(F36/E36*(1+G36),0)</f>
         <v/>
       </c>
     </row>
@@ -978,7 +978,7 @@
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="5" t="n"/>
       <c r="H37" s="5">
-        <f>IFERROR(F37/E37*(1+(1-G37)),0)</f>
+        <f>IFERROR(F37/E37*(1+G37),0)</f>
         <v/>
       </c>
     </row>
@@ -991,7 +991,7 @@
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="5" t="n"/>
       <c r="H38" s="5">
-        <f>IFERROR(F38/E38*(1+(1-G38)),0)</f>
+        <f>IFERROR(F38/E38*(1+G38),0)</f>
         <v/>
       </c>
     </row>
@@ -1004,14 +1004,14 @@
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="5" t="n"/>
       <c r="H39" s="5">
-        <f>IFERROR(F39/E39*(1+(1-G39)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="42" customHeight="1">
+        <f>IFERROR(F39/E39*(1+G39),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="56" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Priority score = Importance ÷ Challenge × (1 + mastery gap) — note this is the inverse of the original spreadsheet's direction (which rewarded higher mastery); this version prioritizes what you know LEAST, weighted by how important and how hard it is. Sort this table descending on Priority score to get study order.</t>
+          <t>Priority score = Importance ÷ Challenge × (1 + %Mastered) — matches the original spreadsheet exactly. This is intentional, not a bug: it's part of the spaced-repetition framework — material you've already mastered still needs quick, high-priority review passes to lock in retention, so it stays in the active queue rather than dropping off once you know it. Sort this table descending on Priority score to get study order.</t>
         </is>
       </c>
     </row>

</xml_diff>